<commit_message>
feat(events): odesílání ohlášky e-mailem z aplikace
Místo stažení XLSX tlačítko „Odeslat ohlášku“ v záložce Lidé pošle ohlášku
přílohou na ANNOUNCEMENT_RECIPIENT (výchozí lef@bosan.cz) a označí ji jako
odeslanou; tlačítko pak zezelená na „Odeslat znovu“. Odeslání se potvrzuje
a chybějící údaje účastníků se vypíšou a odeslání zablokují. Vedoucí
a instruktoři mají v ohlášce vlastní telefon označený „(vlastní)“.

Closes #654

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q4jPMRZWa7My5Q4iuaALib
</commit_message>
<xml_diff>
--- a/backend/assets/annoucement_template.xlsx
+++ b/backend/assets/annoucement_template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
     <t xml:space="preserve">Dětská vodácká skupina Šán</t>
   </si>
@@ -84,12 +84,15 @@
   <si>
     <t xml:space="preserve">Kontakt na blízkou osobu</t>
   </si>
+  <si>
+    <t xml:space="preserve">Kontakt</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts>
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="mm/dd/yy"/>
     <numFmt numFmtId="166" formatCode="m/d/yyyy"/>
@@ -99,7 +102,7 @@
     <numFmt numFmtId="170" formatCode="###\ ##"/>
     <numFmt numFmtId="171" formatCode="000,000,000"/>
   </numFmts>
-  <fonts count="10">
+  <fonts>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -165,8 +168,1064 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial CE"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills>
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -179,8 +1238,1416 @@
         <bgColor rgb="FFFF8080"/>
       </patternFill>
     </fill>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
+    <fill/>
   </fills>
-  <borders count="1">
+  <borders>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -217,7 +2684,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -304,6 +2771,710 @@
     </xf>
     <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="2" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="3" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="6" borderId="4" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="7" borderId="5" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="8" borderId="6" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="9" borderId="7" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="10" borderId="8" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="11" borderId="9" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="12" borderId="10" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="13" borderId="11" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="14" borderId="12" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="15" borderId="13" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="16" borderId="14" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="17" borderId="15" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="18" borderId="16" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="19" borderId="17" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="20" borderId="18" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="21" borderId="19" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="22" borderId="20" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="23" borderId="21" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="24" borderId="22" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="25" borderId="23" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="26" borderId="24" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="27" borderId="25" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="35" fillId="28" borderId="26" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="36" fillId="29" borderId="27" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="37" fillId="30" borderId="28" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="38" fillId="31" borderId="29" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="39" fillId="32" borderId="30" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="40" fillId="33" borderId="31" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="41" fillId="34" borderId="32" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="42" fillId="35" borderId="33" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="43" fillId="36" borderId="34" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="44" fillId="37" borderId="35" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="45" fillId="38" borderId="36" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="46" fillId="39" borderId="37" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="47" fillId="40" borderId="38" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="48" fillId="41" borderId="39" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="49" fillId="42" borderId="40" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="50" fillId="43" borderId="41" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="51" fillId="44" borderId="42" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="52" fillId="45" borderId="43" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="53" fillId="46" borderId="44" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="54" fillId="47" borderId="45" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="55" fillId="48" borderId="46" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="56" fillId="49" borderId="47" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="57" fillId="50" borderId="48" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="58" fillId="51" borderId="49" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="59" fillId="52" borderId="50" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="60" fillId="53" borderId="51" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="61" fillId="54" borderId="52" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="62" fillId="55" borderId="53" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="63" fillId="56" borderId="54" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="64" fillId="57" borderId="55" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="65" fillId="58" borderId="56" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="66" fillId="59" borderId="57" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="67" fillId="60" borderId="58" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="68" fillId="61" borderId="59" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="69" fillId="62" borderId="60" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="70" fillId="63" borderId="61" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="71" fillId="64" borderId="62" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="72" fillId="65" borderId="63" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="73" fillId="66" borderId="64" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="74" fillId="67" borderId="65" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="75" fillId="68" borderId="66" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="76" fillId="69" borderId="67" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="77" fillId="70" borderId="68" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="78" fillId="71" borderId="69" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="79" fillId="72" borderId="70" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="80" fillId="73" borderId="71" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="81" fillId="74" borderId="72" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="82" fillId="75" borderId="73" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="83" fillId="76" borderId="74" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="84" fillId="77" borderId="75" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="85" fillId="78" borderId="76" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="86" fillId="79" borderId="77" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="87" fillId="80" borderId="78" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="88" fillId="81" borderId="79" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="89" fillId="82" borderId="80" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="90" fillId="83" borderId="81" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="91" fillId="84" borderId="82" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="92" fillId="85" borderId="83" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="93" fillId="86" borderId="84" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="94" fillId="87" borderId="85" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="95" fillId="88" borderId="86" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="96" fillId="89" borderId="87" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="97" fillId="90" borderId="88" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="98" fillId="91" borderId="89" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="99" fillId="92" borderId="90" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="100" fillId="93" borderId="91" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="101" fillId="94" borderId="92" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="102" fillId="95" borderId="93" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="103" fillId="96" borderId="94" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="104" fillId="97" borderId="95" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="105" fillId="98" borderId="96" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="106" fillId="99" borderId="97" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="107" fillId="100" borderId="98" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="108" fillId="101" borderId="99" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="109" fillId="102" borderId="100" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="110" fillId="103" borderId="101" xfId="15" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="111" fillId="104" borderId="102" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="112" fillId="105" borderId="103" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="113" fillId="106" borderId="104" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="114" fillId="107" borderId="105" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="115" fillId="108" borderId="106" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="116" fillId="109" borderId="107" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="117" fillId="110" borderId="108" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="118" fillId="111" borderId="109" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="119" fillId="112" borderId="110" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="120" fillId="113" borderId="111" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="121" fillId="114" borderId="112" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="122" fillId="115" borderId="113" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="123" fillId="116" borderId="114" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="124" fillId="117" borderId="115" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="125" fillId="118" borderId="116" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="126" fillId="119" borderId="117" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="127" fillId="120" borderId="118" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="128" fillId="121" borderId="119" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="129" fillId="122" borderId="120" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="130" fillId="123" borderId="121" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="131" fillId="124" borderId="122" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="132" fillId="125" borderId="123" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="133" fillId="126" borderId="124" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="134" fillId="127" borderId="125" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="135" fillId="128" borderId="126" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="136" fillId="129" borderId="127" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="137" fillId="130" borderId="128" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="138" fillId="131" borderId="129" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="139" fillId="132" borderId="130" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="140" fillId="133" borderId="131" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="141" fillId="134" borderId="132" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="142" fillId="135" borderId="133" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="143" fillId="136" borderId="134" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="144" fillId="137" borderId="135" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="145" fillId="138" borderId="136" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="146" fillId="139" borderId="137" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="147" fillId="140" borderId="138" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="148" fillId="141" borderId="139" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="149" fillId="142" borderId="140" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="150" fillId="143" borderId="141" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="151" fillId="144" borderId="142" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="152" fillId="145" borderId="143" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="153" fillId="146" borderId="144" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="154" fillId="147" borderId="145" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="155" fillId="148" borderId="146" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="156" fillId="149" borderId="147" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="157" fillId="150" borderId="148" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="158" fillId="151" borderId="149" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="159" fillId="152" borderId="150" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="160" fillId="153" borderId="151" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="161" fillId="154" borderId="152" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="162" fillId="155" borderId="153" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="163" fillId="156" borderId="154" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="164" fillId="157" borderId="155" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="165" fillId="158" borderId="156" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="166" fillId="159" borderId="157" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="167" fillId="160" borderId="158" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="168" fillId="161" borderId="159" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="169" fillId="162" borderId="160" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="170" fillId="163" borderId="161" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="171" fillId="164" borderId="162" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="172" fillId="165" borderId="163" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="173" fillId="166" borderId="164" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="174" fillId="167" borderId="165" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="175" fillId="168" borderId="166" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="176" fillId="169" borderId="167" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="177" fillId="170" borderId="168" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="178" fillId="171" borderId="169" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="179" fillId="172" borderId="170" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="180" fillId="173" borderId="171" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="181" fillId="174" borderId="172" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="182" fillId="175" borderId="173" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="183" fillId="176" borderId="174" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="184" fillId="177" borderId="175" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="185" fillId="178" borderId="176" xfId="0" applyFont="1" applyBorder="1" applyAlignment="true" applyProtection="true" applyFill="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -598,13 +3769,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H1048576"/>
   <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="1" width="18.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="31.16"/>
+    <col collapsed="false" customWidth="1" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="31.16"/>
+    <col collapsed="false" customWidth="1" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="10.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="12.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="21"/>
@@ -614,7 +3784,7 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="26.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+      <c r="A1" t="s" s="3">
         <v>0</v>
       </c>
       <c r="B1" s="3"/>
@@ -626,12 +3796,12 @@
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F2" s="4"/>
-      <c r="G2" s="5" t="s">
+      <c r="G2" t="s" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="G3" s="5" t="s">
+      <c r="G3" t="s" s="5">
         <v>2</v>
       </c>
     </row>
@@ -645,16 +3815,16 @@
       <c r="E8" s="7"/>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="s">
+      <c r="A10" t="s" s="8">
         <v>3</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s" s="1">
         <v>4</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" t="s" s="5">
         <v>5</v>
       </c>
-      <c r="F10" s="9" t="n">
+      <c r="F10" s="9">
         <v>0</v>
       </c>
     </row>
@@ -662,7 +3832,7 @@
       <c r="A11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+      <c r="A12" t="s" s="5">
         <v>6</v>
       </c>
     </row>
@@ -670,19 +3840,19 @@
       <c r="A13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
+      <c r="A14" t="s" s="5">
         <v>7</v>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B14" s="9">
         <v>0</v>
       </c>
       <c r="C14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+      <c r="A15" t="s" s="5">
         <v>8</v>
       </c>
-      <c r="B15" s="9" t="n">
+      <c r="B15" s="9">
         <v>0</v>
       </c>
       <c r="C15" s="11"/>
@@ -692,18 +3862,18 @@
       <c r="C16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
+      <c r="A17" t="s" s="5">
         <v>9</v>
       </c>
       <c r="C17" s="12"/>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="s">
+      <c r="A18" t="s" s="13">
         <v>10</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="s">
+      <c r="A19" t="s" s="13">
         <v>11</v>
       </c>
       <c r="C19" s="12"/>
@@ -713,7 +3883,7 @@
       <c r="A20" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="13" t="s">
+      <c r="A21" t="s" s="13">
         <v>12</v>
       </c>
     </row>
@@ -721,32 +3891,30 @@
       <c r="A22" s="5"/>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
+      <c r="A23" t="s" s="5">
         <v>13</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="15" t="s">
+      <c r="A24" t="s" s="15">
         <v>14</v>
       </c>
-      <c r="B24" s="15" t="s">
+      <c r="B24" t="s" s="15">
         <v>15</v>
       </c>
-      <c r="C24" s="15" t="s">
+      <c r="C24" t="s" s="15">
         <v>16</v>
       </c>
-      <c r="D24" s="15" t="s">
+      <c r="D24" t="s" s="15">
         <v>17</v>
       </c>
-      <c r="E24" s="15" t="s">
+      <c r="E24" t="s" s="15">
         <v>18</v>
       </c>
-      <c r="F24" s="15" t="s">
-        <v>19</v>
+      <c r="F24" t="s" s="15">
+        <v>21</v>
       </c>
-      <c r="G24" s="15" t="s">
-        <v>20</v>
-      </c>
+      <c r="G24" s="15"/>
       <c r="H24" s="16"/>
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -755,7 +3923,7 @@
       <c r="C25" s="19"/>
       <c r="D25" s="18"/>
       <c r="E25" s="18"/>
-      <c r="F25" s="20"/>
+      <c r="F25" s="22"/>
       <c r="G25" s="21"/>
       <c r="H25" s="16"/>
     </row>
@@ -765,7 +3933,7 @@
       <c r="C26" s="19"/>
       <c r="D26" s="18"/>
       <c r="E26" s="18"/>
-      <c r="F26" s="20"/>
+      <c r="F26" s="23"/>
       <c r="G26" s="21"/>
       <c r="H26" s="16"/>
     </row>
@@ -775,7 +3943,7 @@
       <c r="C27" s="19"/>
       <c r="D27" s="18"/>
       <c r="E27" s="18"/>
-      <c r="F27" s="20"/>
+      <c r="F27" s="24"/>
       <c r="G27" s="21"/>
       <c r="H27" s="16"/>
     </row>
@@ -785,7 +3953,7 @@
       <c r="C28" s="19"/>
       <c r="D28" s="18"/>
       <c r="E28" s="18"/>
-      <c r="F28" s="20"/>
+      <c r="F28" s="25"/>
       <c r="G28" s="21"/>
       <c r="H28" s="16"/>
     </row>
@@ -795,7 +3963,7 @@
       <c r="C29" s="19"/>
       <c r="D29" s="18"/>
       <c r="E29" s="18"/>
-      <c r="F29" s="20"/>
+      <c r="F29" s="26"/>
       <c r="G29" s="21"/>
       <c r="H29" s="16"/>
     </row>
@@ -805,7 +3973,7 @@
       <c r="C30" s="19"/>
       <c r="D30" s="18"/>
       <c r="E30" s="18"/>
-      <c r="F30" s="20"/>
+      <c r="F30" s="27"/>
       <c r="G30" s="21"/>
       <c r="H30" s="16"/>
     </row>
@@ -815,7 +3983,7 @@
       <c r="C31" s="19"/>
       <c r="D31" s="18"/>
       <c r="E31" s="18"/>
-      <c r="F31" s="20"/>
+      <c r="F31" s="28"/>
       <c r="G31" s="21"/>
       <c r="H31" s="16"/>
     </row>
@@ -825,7 +3993,7 @@
       <c r="C32" s="19"/>
       <c r="D32" s="18"/>
       <c r="E32" s="18"/>
-      <c r="F32" s="20"/>
+      <c r="F32" s="29"/>
       <c r="G32" s="21"/>
       <c r="H32" s="16"/>
     </row>
@@ -835,7 +4003,7 @@
       <c r="C33" s="19"/>
       <c r="D33" s="18"/>
       <c r="E33" s="18"/>
-      <c r="F33" s="20"/>
+      <c r="F33" s="30"/>
       <c r="G33" s="21"/>
       <c r="H33" s="16"/>
     </row>
@@ -845,7 +4013,7 @@
       <c r="C34" s="19"/>
       <c r="D34" s="18"/>
       <c r="E34" s="18"/>
-      <c r="F34" s="20"/>
+      <c r="F34" s="31"/>
       <c r="G34" s="21"/>
       <c r="H34" s="16"/>
     </row>
@@ -855,7 +4023,7 @@
       <c r="C35" s="19"/>
       <c r="D35" s="18"/>
       <c r="E35" s="18"/>
-      <c r="F35" s="20"/>
+      <c r="F35" s="32"/>
       <c r="G35" s="21"/>
       <c r="H35" s="16"/>
     </row>
@@ -865,7 +4033,7 @@
       <c r="C36" s="19"/>
       <c r="D36" s="18"/>
       <c r="E36" s="18"/>
-      <c r="F36" s="20"/>
+      <c r="F36" s="33"/>
       <c r="G36" s="21"/>
       <c r="H36" s="16"/>
     </row>
@@ -875,7 +4043,7 @@
       <c r="C37" s="19"/>
       <c r="D37" s="18"/>
       <c r="E37" s="18"/>
-      <c r="F37" s="20"/>
+      <c r="F37" s="34"/>
       <c r="G37" s="21"/>
       <c r="H37" s="16"/>
     </row>
@@ -885,7 +4053,7 @@
       <c r="C38" s="19"/>
       <c r="D38" s="18"/>
       <c r="E38" s="18"/>
-      <c r="F38" s="20"/>
+      <c r="F38" s="35"/>
       <c r="G38" s="21"/>
       <c r="H38" s="16"/>
     </row>
@@ -895,7 +4063,7 @@
       <c r="C39" s="19"/>
       <c r="D39" s="18"/>
       <c r="E39" s="18"/>
-      <c r="F39" s="20"/>
+      <c r="F39" s="36"/>
       <c r="G39" s="21"/>
       <c r="H39" s="16"/>
     </row>
@@ -905,7 +4073,7 @@
       <c r="C40" s="19"/>
       <c r="D40" s="18"/>
       <c r="E40" s="18"/>
-      <c r="F40" s="20"/>
+      <c r="F40" s="37"/>
       <c r="G40" s="21"/>
       <c r="H40" s="16"/>
     </row>
@@ -915,7 +4083,7 @@
       <c r="C41" s="19"/>
       <c r="D41" s="18"/>
       <c r="E41" s="18"/>
-      <c r="F41" s="20"/>
+      <c r="F41" s="38"/>
       <c r="G41" s="21"/>
       <c r="H41" s="16"/>
     </row>
@@ -925,7 +4093,7 @@
       <c r="C42" s="19"/>
       <c r="D42" s="18"/>
       <c r="E42" s="18"/>
-      <c r="F42" s="20"/>
+      <c r="F42" s="39"/>
       <c r="G42" s="21"/>
       <c r="H42" s="16"/>
     </row>
@@ -935,7 +4103,7 @@
       <c r="C43" s="19"/>
       <c r="D43" s="18"/>
       <c r="E43" s="18"/>
-      <c r="F43" s="20"/>
+      <c r="F43" s="40"/>
       <c r="G43" s="21"/>
     </row>
     <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -944,7 +4112,7 @@
       <c r="C44" s="19"/>
       <c r="D44" s="18"/>
       <c r="E44" s="18"/>
-      <c r="F44" s="20"/>
+      <c r="F44" s="41"/>
       <c r="G44" s="21"/>
     </row>
     <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -953,7 +4121,7 @@
       <c r="C45" s="19"/>
       <c r="D45" s="18"/>
       <c r="E45" s="18"/>
-      <c r="F45" s="20"/>
+      <c r="F45" s="42"/>
       <c r="G45" s="21"/>
     </row>
     <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -962,7 +4130,7 @@
       <c r="C46" s="19"/>
       <c r="D46" s="18"/>
       <c r="E46" s="18"/>
-      <c r="F46" s="20"/>
+      <c r="F46" s="43"/>
       <c r="G46" s="21"/>
     </row>
     <row r="47" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -971,7 +4139,7 @@
       <c r="C47" s="19"/>
       <c r="D47" s="18"/>
       <c r="E47" s="18"/>
-      <c r="F47" s="20"/>
+      <c r="F47" s="44"/>
       <c r="G47" s="21"/>
     </row>
     <row r="48" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -980,7 +4148,7 @@
       <c r="C48" s="19"/>
       <c r="D48" s="18"/>
       <c r="E48" s="18"/>
-      <c r="F48" s="20"/>
+      <c r="F48" s="45"/>
       <c r="G48" s="21"/>
     </row>
     <row r="49" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -989,7 +4157,7 @@
       <c r="C49" s="19"/>
       <c r="D49" s="18"/>
       <c r="E49" s="18"/>
-      <c r="F49" s="20"/>
+      <c r="F49" s="46"/>
       <c r="G49" s="21"/>
     </row>
     <row r="50" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -998,7 +4166,7 @@
       <c r="C50" s="19"/>
       <c r="D50" s="18"/>
       <c r="E50" s="18"/>
-      <c r="F50" s="20"/>
+      <c r="F50" s="47"/>
       <c r="G50" s="21"/>
     </row>
     <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1007,7 +4175,7 @@
       <c r="C51" s="19"/>
       <c r="D51" s="18"/>
       <c r="E51" s="18"/>
-      <c r="F51" s="20"/>
+      <c r="F51" s="48"/>
       <c r="G51" s="21"/>
     </row>
     <row r="52" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1016,7 +4184,7 @@
       <c r="C52" s="19"/>
       <c r="D52" s="18"/>
       <c r="E52" s="18"/>
-      <c r="F52" s="20"/>
+      <c r="F52" s="49"/>
       <c r="G52" s="21"/>
     </row>
     <row r="53" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1025,7 +4193,7 @@
       <c r="C53" s="19"/>
       <c r="D53" s="18"/>
       <c r="E53" s="18"/>
-      <c r="F53" s="20"/>
+      <c r="F53" s="50"/>
       <c r="G53" s="21"/>
     </row>
     <row r="54" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1034,7 +4202,7 @@
       <c r="C54" s="19"/>
       <c r="D54" s="18"/>
       <c r="E54" s="18"/>
-      <c r="F54" s="20"/>
+      <c r="F54" s="51"/>
       <c r="G54" s="21"/>
     </row>
     <row r="55" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1043,7 +4211,7 @@
       <c r="C55" s="19"/>
       <c r="D55" s="18"/>
       <c r="E55" s="18"/>
-      <c r="F55" s="20"/>
+      <c r="F55" s="52"/>
       <c r="G55" s="21"/>
     </row>
     <row r="56" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1052,7 +4220,7 @@
       <c r="C56" s="19"/>
       <c r="D56" s="18"/>
       <c r="E56" s="18"/>
-      <c r="F56" s="20"/>
+      <c r="F56" s="53"/>
       <c r="G56" s="21"/>
     </row>
     <row r="57" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1061,7 +4229,7 @@
       <c r="C57" s="19"/>
       <c r="D57" s="18"/>
       <c r="E57" s="18"/>
-      <c r="F57" s="20"/>
+      <c r="F57" s="54"/>
       <c r="G57" s="21"/>
     </row>
     <row r="58" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1070,7 +4238,7 @@
       <c r="C58" s="19"/>
       <c r="D58" s="18"/>
       <c r="E58" s="18"/>
-      <c r="F58" s="20"/>
+      <c r="F58" s="55"/>
       <c r="G58" s="21"/>
     </row>
     <row r="59" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1079,7 +4247,7 @@
       <c r="C59" s="19"/>
       <c r="D59" s="18"/>
       <c r="E59" s="18"/>
-      <c r="F59" s="20"/>
+      <c r="F59" s="56"/>
       <c r="G59" s="21"/>
     </row>
     <row r="60" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1088,7 +4256,7 @@
       <c r="C60" s="19"/>
       <c r="D60" s="18"/>
       <c r="E60" s="18"/>
-      <c r="F60" s="20"/>
+      <c r="F60" s="57"/>
       <c r="G60" s="21"/>
     </row>
     <row r="61" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1097,7 +4265,7 @@
       <c r="C61" s="19"/>
       <c r="D61" s="18"/>
       <c r="E61" s="18"/>
-      <c r="F61" s="20"/>
+      <c r="F61" s="58"/>
       <c r="G61" s="21"/>
     </row>
     <row r="62" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1106,7 +4274,7 @@
       <c r="C62" s="19"/>
       <c r="D62" s="18"/>
       <c r="E62" s="18"/>
-      <c r="F62" s="20"/>
+      <c r="F62" s="59"/>
       <c r="G62" s="21"/>
     </row>
     <row r="63" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1115,7 +4283,7 @@
       <c r="C63" s="19"/>
       <c r="D63" s="18"/>
       <c r="E63" s="18"/>
-      <c r="F63" s="20"/>
+      <c r="F63" s="60"/>
       <c r="G63" s="21"/>
     </row>
     <row r="64" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1124,7 +4292,7 @@
       <c r="C64" s="19"/>
       <c r="D64" s="18"/>
       <c r="E64" s="18"/>
-      <c r="F64" s="20"/>
+      <c r="F64" s="61"/>
       <c r="G64" s="21"/>
     </row>
     <row r="65" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1133,7 +4301,7 @@
       <c r="C65" s="19"/>
       <c r="D65" s="18"/>
       <c r="E65" s="18"/>
-      <c r="F65" s="20"/>
+      <c r="F65" s="62"/>
       <c r="G65" s="21"/>
     </row>
     <row r="66" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1142,7 +4310,7 @@
       <c r="C66" s="19"/>
       <c r="D66" s="18"/>
       <c r="E66" s="18"/>
-      <c r="F66" s="20"/>
+      <c r="F66" s="63"/>
       <c r="G66" s="21"/>
     </row>
     <row r="67" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1151,7 +4319,7 @@
       <c r="C67" s="19"/>
       <c r="D67" s="18"/>
       <c r="E67" s="18"/>
-      <c r="F67" s="20"/>
+      <c r="F67" s="64"/>
       <c r="G67" s="21"/>
     </row>
     <row r="68" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1160,7 +4328,7 @@
       <c r="C68" s="19"/>
       <c r="D68" s="18"/>
       <c r="E68" s="18"/>
-      <c r="F68" s="20"/>
+      <c r="F68" s="65"/>
       <c r="G68" s="21"/>
     </row>
     <row r="69" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1169,7 +4337,7 @@
       <c r="C69" s="19"/>
       <c r="D69" s="18"/>
       <c r="E69" s="18"/>
-      <c r="F69" s="20"/>
+      <c r="F69" s="66"/>
       <c r="G69" s="21"/>
     </row>
     <row r="70" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1178,7 +4346,7 @@
       <c r="C70" s="19"/>
       <c r="D70" s="18"/>
       <c r="E70" s="18"/>
-      <c r="F70" s="20"/>
+      <c r="F70" s="67"/>
       <c r="G70" s="21"/>
     </row>
     <row r="71" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1187,7 +4355,7 @@
       <c r="C71" s="19"/>
       <c r="D71" s="18"/>
       <c r="E71" s="18"/>
-      <c r="F71" s="20"/>
+      <c r="F71" s="68"/>
       <c r="G71" s="21"/>
     </row>
     <row r="72" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1196,7 +4364,7 @@
       <c r="C72" s="19"/>
       <c r="D72" s="18"/>
       <c r="E72" s="18"/>
-      <c r="F72" s="20"/>
+      <c r="F72" s="69"/>
       <c r="G72" s="21"/>
     </row>
     <row r="73" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1205,7 +4373,7 @@
       <c r="C73" s="19"/>
       <c r="D73" s="18"/>
       <c r="E73" s="18"/>
-      <c r="F73" s="20"/>
+      <c r="F73" s="70"/>
       <c r="G73" s="21"/>
     </row>
     <row r="74" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1214,7 +4382,7 @@
       <c r="C74" s="19"/>
       <c r="D74" s="18"/>
       <c r="E74" s="18"/>
-      <c r="F74" s="20"/>
+      <c r="F74" s="71"/>
       <c r="G74" s="21"/>
     </row>
     <row r="75" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1223,7 +4391,7 @@
       <c r="C75" s="19"/>
       <c r="D75" s="18"/>
       <c r="E75" s="18"/>
-      <c r="F75" s="20"/>
+      <c r="F75" s="72"/>
       <c r="G75" s="21"/>
     </row>
     <row r="76" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1232,7 +4400,7 @@
       <c r="C76" s="19"/>
       <c r="D76" s="18"/>
       <c r="E76" s="18"/>
-      <c r="F76" s="20"/>
+      <c r="F76" s="73"/>
       <c r="G76" s="21"/>
     </row>
     <row r="77" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1241,7 +4409,7 @@
       <c r="C77" s="19"/>
       <c r="D77" s="18"/>
       <c r="E77" s="18"/>
-      <c r="F77" s="20"/>
+      <c r="F77" s="74"/>
       <c r="G77" s="21"/>
     </row>
     <row r="78" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1250,7 +4418,7 @@
       <c r="C78" s="19"/>
       <c r="D78" s="18"/>
       <c r="E78" s="18"/>
-      <c r="F78" s="20"/>
+      <c r="F78" s="75"/>
       <c r="G78" s="21"/>
     </row>
     <row r="79" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1259,7 +4427,7 @@
       <c r="C79" s="19"/>
       <c r="D79" s="18"/>
       <c r="E79" s="18"/>
-      <c r="F79" s="20"/>
+      <c r="F79" s="76"/>
       <c r="G79" s="21"/>
     </row>
     <row r="80" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1268,7 +4436,7 @@
       <c r="C80" s="19"/>
       <c r="D80" s="18"/>
       <c r="E80" s="18"/>
-      <c r="F80" s="20"/>
+      <c r="F80" s="77"/>
       <c r="G80" s="21"/>
     </row>
     <row r="81" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1277,7 +4445,7 @@
       <c r="C81" s="19"/>
       <c r="D81" s="18"/>
       <c r="E81" s="18"/>
-      <c r="F81" s="20"/>
+      <c r="F81" s="78"/>
       <c r="G81" s="21"/>
     </row>
     <row r="82" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1286,7 +4454,7 @@
       <c r="C82" s="19"/>
       <c r="D82" s="18"/>
       <c r="E82" s="18"/>
-      <c r="F82" s="20"/>
+      <c r="F82" s="79"/>
       <c r="G82" s="21"/>
     </row>
     <row r="83" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1295,7 +4463,7 @@
       <c r="C83" s="19"/>
       <c r="D83" s="18"/>
       <c r="E83" s="18"/>
-      <c r="F83" s="20"/>
+      <c r="F83" s="80"/>
       <c r="G83" s="21"/>
     </row>
     <row r="84" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1304,7 +4472,7 @@
       <c r="C84" s="19"/>
       <c r="D84" s="18"/>
       <c r="E84" s="18"/>
-      <c r="F84" s="20"/>
+      <c r="F84" s="81"/>
       <c r="G84" s="21"/>
     </row>
     <row r="85" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1313,7 +4481,7 @@
       <c r="C85" s="19"/>
       <c r="D85" s="18"/>
       <c r="E85" s="18"/>
-      <c r="F85" s="20"/>
+      <c r="F85" s="82"/>
       <c r="G85" s="21"/>
     </row>
     <row r="86" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1322,7 +4490,7 @@
       <c r="C86" s="19"/>
       <c r="D86" s="18"/>
       <c r="E86" s="18"/>
-      <c r="F86" s="20"/>
+      <c r="F86" s="83"/>
       <c r="G86" s="21"/>
     </row>
     <row r="87" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1331,7 +4499,7 @@
       <c r="C87" s="19"/>
       <c r="D87" s="18"/>
       <c r="E87" s="18"/>
-      <c r="F87" s="20"/>
+      <c r="F87" s="84"/>
       <c r="G87" s="21"/>
     </row>
     <row r="88" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1340,7 +4508,7 @@
       <c r="C88" s="19"/>
       <c r="D88" s="18"/>
       <c r="E88" s="18"/>
-      <c r="F88" s="20"/>
+      <c r="F88" s="85"/>
       <c r="G88" s="21"/>
     </row>
     <row r="89" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1349,7 +4517,7 @@
       <c r="C89" s="19"/>
       <c r="D89" s="18"/>
       <c r="E89" s="18"/>
-      <c r="F89" s="20"/>
+      <c r="F89" s="86"/>
       <c r="G89" s="21"/>
     </row>
     <row r="90" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1358,7 +4526,7 @@
       <c r="C90" s="19"/>
       <c r="D90" s="18"/>
       <c r="E90" s="18"/>
-      <c r="F90" s="20"/>
+      <c r="F90" s="87"/>
       <c r="G90" s="21"/>
     </row>
     <row r="91" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1367,7 +4535,7 @@
       <c r="C91" s="19"/>
       <c r="D91" s="18"/>
       <c r="E91" s="18"/>
-      <c r="F91" s="20"/>
+      <c r="F91" s="88"/>
       <c r="G91" s="21"/>
     </row>
     <row r="92" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1376,7 +4544,7 @@
       <c r="C92" s="19"/>
       <c r="D92" s="18"/>
       <c r="E92" s="18"/>
-      <c r="F92" s="20"/>
+      <c r="F92" s="89"/>
       <c r="G92" s="21"/>
     </row>
     <row r="93" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1385,7 +4553,7 @@
       <c r="C93" s="19"/>
       <c r="D93" s="18"/>
       <c r="E93" s="18"/>
-      <c r="F93" s="20"/>
+      <c r="F93" s="90"/>
       <c r="G93" s="21"/>
     </row>
     <row r="94" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1394,7 +4562,7 @@
       <c r="C94" s="19"/>
       <c r="D94" s="18"/>
       <c r="E94" s="18"/>
-      <c r="F94" s="20"/>
+      <c r="F94" s="91"/>
       <c r="G94" s="21"/>
     </row>
     <row r="95" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1403,7 +4571,7 @@
       <c r="C95" s="19"/>
       <c r="D95" s="18"/>
       <c r="E95" s="18"/>
-      <c r="F95" s="20"/>
+      <c r="F95" s="92"/>
       <c r="G95" s="21"/>
     </row>
     <row r="96" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1412,7 +4580,7 @@
       <c r="C96" s="19"/>
       <c r="D96" s="18"/>
       <c r="E96" s="18"/>
-      <c r="F96" s="20"/>
+      <c r="F96" s="93"/>
       <c r="G96" s="21"/>
     </row>
     <row r="97" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1421,7 +4589,7 @@
       <c r="C97" s="19"/>
       <c r="D97" s="18"/>
       <c r="E97" s="18"/>
-      <c r="F97" s="20"/>
+      <c r="F97" s="94"/>
       <c r="G97" s="21"/>
     </row>
     <row r="98" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1430,7 +4598,7 @@
       <c r="C98" s="19"/>
       <c r="D98" s="18"/>
       <c r="E98" s="18"/>
-      <c r="F98" s="20"/>
+      <c r="F98" s="95"/>
       <c r="G98" s="21"/>
     </row>
     <row r="99" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1439,7 +4607,7 @@
       <c r="C99" s="19"/>
       <c r="D99" s="18"/>
       <c r="E99" s="18"/>
-      <c r="F99" s="20"/>
+      <c r="F99" s="96"/>
       <c r="G99" s="21"/>
     </row>
     <row r="100" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1448,7 +4616,7 @@
       <c r="C100" s="19"/>
       <c r="D100" s="18"/>
       <c r="E100" s="18"/>
-      <c r="F100" s="20"/>
+      <c r="F100" s="97"/>
       <c r="G100" s="21"/>
     </row>
     <row r="101" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1457,7 +4625,7 @@
       <c r="C101" s="19"/>
       <c r="D101" s="18"/>
       <c r="E101" s="18"/>
-      <c r="F101" s="20"/>
+      <c r="F101" s="98"/>
       <c r="G101" s="21"/>
     </row>
     <row r="102" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1466,7 +4634,7 @@
       <c r="C102" s="19"/>
       <c r="D102" s="18"/>
       <c r="E102" s="18"/>
-      <c r="F102" s="20"/>
+      <c r="F102" s="99"/>
       <c r="G102" s="21"/>
     </row>
     <row r="103" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1475,7 +4643,7 @@
       <c r="C103" s="19"/>
       <c r="D103" s="18"/>
       <c r="E103" s="18"/>
-      <c r="F103" s="20"/>
+      <c r="F103" s="100"/>
       <c r="G103" s="21"/>
     </row>
     <row r="104" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1484,7 +4652,7 @@
       <c r="C104" s="19"/>
       <c r="D104" s="18"/>
       <c r="E104" s="18"/>
-      <c r="F104" s="20"/>
+      <c r="F104" s="101"/>
       <c r="G104" s="21"/>
     </row>
     <row r="105" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1493,7 +4661,7 @@
       <c r="C105" s="19"/>
       <c r="D105" s="18"/>
       <c r="E105" s="18"/>
-      <c r="F105" s="20"/>
+      <c r="F105" s="102"/>
       <c r="G105" s="21"/>
     </row>
     <row r="106" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1502,7 +4670,7 @@
       <c r="C106" s="19"/>
       <c r="D106" s="18"/>
       <c r="E106" s="18"/>
-      <c r="F106" s="20"/>
+      <c r="F106" s="103"/>
       <c r="G106" s="21"/>
     </row>
     <row r="107" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1511,7 +4679,7 @@
       <c r="C107" s="19"/>
       <c r="D107" s="18"/>
       <c r="E107" s="18"/>
-      <c r="F107" s="20"/>
+      <c r="F107" s="104"/>
       <c r="G107" s="21"/>
     </row>
     <row r="108" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1520,7 +4688,7 @@
       <c r="C108" s="19"/>
       <c r="D108" s="18"/>
       <c r="E108" s="18"/>
-      <c r="F108" s="20"/>
+      <c r="F108" s="105"/>
       <c r="G108" s="21"/>
     </row>
     <row r="109" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1529,7 +4697,7 @@
       <c r="C109" s="19"/>
       <c r="D109" s="18"/>
       <c r="E109" s="18"/>
-      <c r="F109" s="20"/>
+      <c r="F109" s="106"/>
       <c r="G109" s="21"/>
     </row>
     <row r="110" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1538,7 +4706,7 @@
       <c r="C110" s="19"/>
       <c r="D110" s="18"/>
       <c r="E110" s="18"/>
-      <c r="F110" s="20"/>
+      <c r="F110" s="107"/>
       <c r="G110" s="21"/>
     </row>
     <row r="111" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1547,7 +4715,7 @@
       <c r="C111" s="19"/>
       <c r="D111" s="18"/>
       <c r="E111" s="18"/>
-      <c r="F111" s="20"/>
+      <c r="F111" s="108"/>
       <c r="G111" s="21"/>
     </row>
     <row r="112" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1556,7 +4724,7 @@
       <c r="C112" s="19"/>
       <c r="D112" s="18"/>
       <c r="E112" s="18"/>
-      <c r="F112" s="20"/>
+      <c r="F112" s="109"/>
       <c r="G112" s="21"/>
     </row>
     <row r="113" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1565,7 +4733,7 @@
       <c r="C113" s="19"/>
       <c r="D113" s="18"/>
       <c r="E113" s="18"/>
-      <c r="F113" s="20"/>
+      <c r="F113" s="110"/>
       <c r="G113" s="21"/>
     </row>
     <row r="114" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1574,7 +4742,7 @@
       <c r="C114" s="19"/>
       <c r="D114" s="18"/>
       <c r="E114" s="18"/>
-      <c r="F114" s="20"/>
+      <c r="F114" s="111"/>
       <c r="G114" s="21"/>
     </row>
     <row r="115" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1583,7 +4751,7 @@
       <c r="C115" s="19"/>
       <c r="D115" s="18"/>
       <c r="E115" s="18"/>
-      <c r="F115" s="20"/>
+      <c r="F115" s="112"/>
       <c r="G115" s="21"/>
     </row>
     <row r="116" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1592,7 +4760,7 @@
       <c r="C116" s="19"/>
       <c r="D116" s="18"/>
       <c r="E116" s="18"/>
-      <c r="F116" s="20"/>
+      <c r="F116" s="113"/>
       <c r="G116" s="21"/>
     </row>
     <row r="117" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1601,7 +4769,7 @@
       <c r="C117" s="19"/>
       <c r="D117" s="18"/>
       <c r="E117" s="18"/>
-      <c r="F117" s="20"/>
+      <c r="F117" s="114"/>
       <c r="G117" s="21"/>
     </row>
     <row r="118" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1610,7 +4778,7 @@
       <c r="C118" s="19"/>
       <c r="D118" s="18"/>
       <c r="E118" s="18"/>
-      <c r="F118" s="20"/>
+      <c r="F118" s="115"/>
       <c r="G118" s="21"/>
     </row>
     <row r="119" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1619,7 +4787,7 @@
       <c r="C119" s="19"/>
       <c r="D119" s="18"/>
       <c r="E119" s="18"/>
-      <c r="F119" s="20"/>
+      <c r="F119" s="116"/>
       <c r="G119" s="21"/>
     </row>
     <row r="120" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1628,7 +4796,7 @@
       <c r="C120" s="19"/>
       <c r="D120" s="18"/>
       <c r="E120" s="18"/>
-      <c r="F120" s="20"/>
+      <c r="F120" s="117"/>
       <c r="G120" s="21"/>
     </row>
     <row r="121" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1637,7 +4805,7 @@
       <c r="C121" s="19"/>
       <c r="D121" s="18"/>
       <c r="E121" s="18"/>
-      <c r="F121" s="20"/>
+      <c r="F121" s="118"/>
       <c r="G121" s="21"/>
     </row>
     <row r="122" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1646,7 +4814,7 @@
       <c r="C122" s="19"/>
       <c r="D122" s="18"/>
       <c r="E122" s="18"/>
-      <c r="F122" s="20"/>
+      <c r="F122" s="119"/>
       <c r="G122" s="21"/>
     </row>
     <row r="123" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1655,7 +4823,7 @@
       <c r="C123" s="19"/>
       <c r="D123" s="18"/>
       <c r="E123" s="18"/>
-      <c r="F123" s="20"/>
+      <c r="F123" s="120"/>
       <c r="G123" s="21"/>
     </row>
     <row r="124" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1664,7 +4832,7 @@
       <c r="C124" s="19"/>
       <c r="D124" s="18"/>
       <c r="E124" s="18"/>
-      <c r="F124" s="20"/>
+      <c r="F124" s="121"/>
       <c r="G124" s="21"/>
     </row>
     <row r="125" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1673,8 +4841,233 @@
       <c r="C125" s="19"/>
       <c r="D125" s="18"/>
       <c r="E125" s="18"/>
-      <c r="F125" s="20"/>
+      <c r="F125" s="122"/>
       <c r="G125" s="21"/>
+    </row>
+    <row r="126">
+      <c r="F126" s="123"/>
+    </row>
+    <row r="127">
+      <c r="F127" s="124"/>
+    </row>
+    <row r="128">
+      <c r="F128" s="125"/>
+    </row>
+    <row r="129">
+      <c r="F129" s="126"/>
+    </row>
+    <row r="130">
+      <c r="F130" s="127"/>
+    </row>
+    <row r="131">
+      <c r="F131" s="128"/>
+    </row>
+    <row r="132">
+      <c r="F132" s="129"/>
+    </row>
+    <row r="133">
+      <c r="F133" s="130"/>
+    </row>
+    <row r="134">
+      <c r="F134" s="131"/>
+    </row>
+    <row r="135">
+      <c r="F135" s="132"/>
+    </row>
+    <row r="136">
+      <c r="F136" s="133"/>
+    </row>
+    <row r="137">
+      <c r="F137" s="134"/>
+    </row>
+    <row r="138">
+      <c r="F138" s="135"/>
+    </row>
+    <row r="139">
+      <c r="F139" s="136"/>
+    </row>
+    <row r="140">
+      <c r="F140" s="137"/>
+    </row>
+    <row r="141">
+      <c r="F141" s="138"/>
+    </row>
+    <row r="142">
+      <c r="F142" s="139"/>
+    </row>
+    <row r="143">
+      <c r="F143" s="140"/>
+    </row>
+    <row r="144">
+      <c r="F144" s="141"/>
+    </row>
+    <row r="145">
+      <c r="F145" s="142"/>
+    </row>
+    <row r="146">
+      <c r="F146" s="143"/>
+    </row>
+    <row r="147">
+      <c r="F147" s="144"/>
+    </row>
+    <row r="148">
+      <c r="F148" s="145"/>
+    </row>
+    <row r="149">
+      <c r="F149" s="146"/>
+    </row>
+    <row r="150">
+      <c r="F150" s="147"/>
+    </row>
+    <row r="151">
+      <c r="F151" s="148"/>
+    </row>
+    <row r="152">
+      <c r="F152" s="149"/>
+    </row>
+    <row r="153">
+      <c r="F153" s="150"/>
+    </row>
+    <row r="154">
+      <c r="F154" s="151"/>
+    </row>
+    <row r="155">
+      <c r="F155" s="152"/>
+    </row>
+    <row r="156">
+      <c r="F156" s="153"/>
+    </row>
+    <row r="157">
+      <c r="F157" s="154"/>
+    </row>
+    <row r="158">
+      <c r="F158" s="155"/>
+    </row>
+    <row r="159">
+      <c r="F159" s="156"/>
+    </row>
+    <row r="160">
+      <c r="F160" s="157"/>
+    </row>
+    <row r="161">
+      <c r="F161" s="158"/>
+    </row>
+    <row r="162">
+      <c r="F162" s="159"/>
+    </row>
+    <row r="163">
+      <c r="F163" s="160"/>
+    </row>
+    <row r="164">
+      <c r="F164" s="161"/>
+    </row>
+    <row r="165">
+      <c r="F165" s="162"/>
+    </row>
+    <row r="166">
+      <c r="F166" s="163"/>
+    </row>
+    <row r="167">
+      <c r="F167" s="164"/>
+    </row>
+    <row r="168">
+      <c r="F168" s="165"/>
+    </row>
+    <row r="169">
+      <c r="F169" s="166"/>
+    </row>
+    <row r="170">
+      <c r="F170" s="167"/>
+    </row>
+    <row r="171">
+      <c r="F171" s="168"/>
+    </row>
+    <row r="172">
+      <c r="F172" s="169"/>
+    </row>
+    <row r="173">
+      <c r="F173" s="170"/>
+    </row>
+    <row r="174">
+      <c r="F174" s="171"/>
+    </row>
+    <row r="175">
+      <c r="F175" s="172"/>
+    </row>
+    <row r="176">
+      <c r="F176" s="173"/>
+    </row>
+    <row r="177">
+      <c r="F177" s="174"/>
+    </row>
+    <row r="178">
+      <c r="F178" s="175"/>
+    </row>
+    <row r="179">
+      <c r="F179" s="176"/>
+    </row>
+    <row r="180">
+      <c r="F180" s="177"/>
+    </row>
+    <row r="181">
+      <c r="F181" s="178"/>
+    </row>
+    <row r="182">
+      <c r="F182" s="179"/>
+    </row>
+    <row r="183">
+      <c r="F183" s="180"/>
+    </row>
+    <row r="184">
+      <c r="F184" s="181"/>
+    </row>
+    <row r="185">
+      <c r="F185" s="182"/>
+    </row>
+    <row r="186">
+      <c r="F186" s="183"/>
+    </row>
+    <row r="187">
+      <c r="F187" s="184"/>
+    </row>
+    <row r="188">
+      <c r="F188" s="185"/>
+    </row>
+    <row r="189">
+      <c r="F189" s="186"/>
+    </row>
+    <row r="190">
+      <c r="F190" s="187"/>
+    </row>
+    <row r="191">
+      <c r="F191" s="188"/>
+    </row>
+    <row r="192">
+      <c r="F192" s="189"/>
+    </row>
+    <row r="193">
+      <c r="F193" s="190"/>
+    </row>
+    <row r="194">
+      <c r="F194" s="191"/>
+    </row>
+    <row r="195">
+      <c r="F195" s="192"/>
+    </row>
+    <row r="196">
+      <c r="F196" s="193"/>
+    </row>
+    <row r="197">
+      <c r="F197" s="194"/>
+    </row>
+    <row r="198">
+      <c r="F198" s="195"/>
+    </row>
+    <row r="199">
+      <c r="F199" s="196"/>
+    </row>
+    <row r="200">
+      <c r="F200" s="197"/>
     </row>
     <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>